<commit_message>
WIP snapshot: Levels 3-4 lessons still in review (not final)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/03-data-analysis/02-data-validation-conditional-formatting/3.2-data-validation-conditional-formatting.xlsx
+++ b/03-data-analysis/02-data-validation-conditional-formatting/3.2-data-validation-conditional-formatting.xlsx
@@ -813,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C35"/>
+  <dimension ref="B2:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -966,7 +966,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="33" customHeight="1">
+    <row r="18" ht="48" customHeight="1">
       <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Note</t>
@@ -974,7 +974,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Part A of the practice uses IntakeLog and Lists. Part B uses Labs, Supplies, and Census. The bonus uses Huddle and NovCensus.</t>
+          <t>Part A of the practice uses IntakeLog and Lists (the drop-down source lists). Part B uses Labs, Supplies, and Census. The bonus uses Huddle (the board you format) and NovCensus (the data behind its unit card).</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>ReportDate (12/31/2025) and ExpiringWindowDays (90) are named cells on the Lists sheet. Use the names in your rules.</t>
+          <t>The data sheets are Excel Tables, so their filter arrows are already on. Use them to filter by color and count what your rules highlight.</t>
         </is>
       </c>
     </row>
@@ -998,153 +998,165 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
+          <t>ReportDate (12/31/2025) and ExpiringWindowDays (90) are named cells on the Lists sheet. Use the names in your rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="33" customHeight="1">
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
           <t>Circle Invalid Data circles disappear when you save or close the file. They are a checking tool, not formatting.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Color legend</t>
         </is>
       </c>
-      <c r="C22" s="5" t="n"/>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="9" t="inlineStr">
+      <c r="C23" s="5" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Yellow cell</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Your answer goes here.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="10" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Gray cell</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Pre-filled summary formula — it reads the work you did on another sheet.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="11" t="inlineStr">
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>✔ Correct</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Your answer matches the key.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="B26" s="12" t="inlineStr">
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>✘ Not yet</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Not matching yet — check the hint and try again.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Sheets in this workbook</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n"/>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>IntakeLog</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Data: 50 rows — Excel Table 'tblIntake'</t>
-        </is>
-      </c>
+      <c r="C29" s="5" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Labs</t>
+          <t>IntakeLog</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Data: 321 rows — Excel Table 'tblLabs'</t>
+          <t>Data: 50 rows — Excel Table 'tblIntake'</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Supplies</t>
+          <t>Labs</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Data: 257 rows — Excel Table 'tblSupplies'</t>
+          <t>Data: 321 rows — Excel Table 'tblLabs'</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Census</t>
+          <t>Supplies</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Data: 61 rows — Excel Table 'tblCensus'</t>
+          <t>Data: 257 rows — Excel Table 'tblSupplies'</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="8" t="inlineStr">
         <is>
+          <t>Census</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Data: 61 rows — Excel Table 'tblCensus'</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
           <t>NovCensus</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Data: 450 rows — Excel Table 'tblNovCensus'</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="48" customHeight="1">
-      <c r="B34" s="8" t="inlineStr">
+    <row r="35" ht="48" customHeight="1">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>About the data</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>A December 2025 Patient Access intake log with entry errors, STAT lab results from the three ICUs (Jul–Dec 2025), the system supply inventory (12/31/2025 snapshot), and Medical-Surgical 5 East's daily census (Nov–Dec 2025). The bonus adds a bed-huddle board for every inpatient unit.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="B35" s="8" t="inlineStr">
+    <row r="36" ht="18" customHeight="1">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Disclaimer</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>All people, places, and numbers are synthetic and fictional. Not clinical guidance.</t>
         </is>
@@ -12240,7 +12252,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="321" customHeight="1">
+    <row r="10" ht="336" customHeight="1">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>6</t>
@@ -12256,7 +12268,7 @@
       </c>
       <c r="D10" s="46" t="inlineStr">
         <is>
-          <t>1. On Lists, select E1:E16 and choose Formulas → Create from Selection, tick only Top row, and click OK. Repeat for F1:F5, G1:G6, H1:H7. Formulas → Name Manager (Ctrl + F3) now lists four names such as Cedar_Ridge_Medical_Center.
+          <t>1. On Lists, select E1:E16 and choose Formulas → Create from Selection, tick only Top row, and click OK. Repeat for F1:F5, G1:G6, H1:H7. Formulas → Name Manager (Windows: Ctrl + F3) now includes four new names, such as Cedar_Ridge_Medical_Center.
 2. Select H2:H51 on IntakeLog → Data Validation → List, Source =Lists!$C$2:$C$5.
 3. Select I2:I51 with I2 active → Data Validation → List, Source =INDIRECT(SUBSTITUTE($H2," ","_")). Click OK.
 4. Click the arrow on Data → Data Validation, then Circle Invalid Data. (Clear Validation Circles removes them.) You see 4 circles.
@@ -12313,7 +12325,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Labs, TATMin (L2:L322): turnaround minutes from specimen collection to result. Apply Top/Bottom Rules → Top 10 Items. What is the smallest TAT that your rule highlights?</t>
+          <t>Labs, TATMin (L2:L322): turnaround minutes from specimen collection to result. Apply Top/Bottom Rules → Top 10 Items. What is the smallest TAT that your rule highlights? Enter it in minutes.</t>
         </is>
       </c>
       <c r="C12" s="45" t="n">
@@ -12337,7 +12349,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="171" customHeight="1">
+    <row r="13" ht="231" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
           <t>9</t>
@@ -12345,7 +12357,7 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Supplies, PctOfPar (K2:K258) = QtyOnHand ÷ ParLevel. Add Data Bars, then edit the rule so Minimum is Number 0 and Maximum is Number 1. A full bar now means "stocked to par." How many items show a completely full bar?</t>
+          <t>Supplies, PctOfPar (K2:K258) is QtyOnHand ÷ ParLevel. Add Data Bars, then edit the rule so Minimum is Type Number, Value 0 and Maximum is Type Number, Value 1. A full bar now means "stocked to par or above." How many items show a full bar?</t>
         </is>
       </c>
       <c r="C13" s="45" t="n">
@@ -12356,7 +12368,7 @@
           <t>1. On Supplies, select K2:K258.
 2. Home → Conditional Formatting → Data Bars and pick any fill.
 3. Conditional Formatting → Manage Rules → Edit Rule. Set Minimum Type = Number, Value = 0, and Maximum Type = Number, Value = 1. Click OK twice.
-4. Count the full bars: 78.
+4. A data bar isn't a fill color, so Filter by Color can't find the full ones. Count them with the formula below instead, because every value of 1 (100%) or more gets a full bar: 78.
 Equivalent formula: =COUNTIF(Supplies!K2:K258,"&gt;=1")</t>
         </is>
       </c>
@@ -12370,7 +12382,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="171" customHeight="1">
+    <row r="14" ht="216" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>10</t>
@@ -12389,6 +12401,7 @@
           <t>1. On Census, select F2:F62.
 2. Home → Conditional Formatting → Color Scales → Red - Yellow - Green Color Scale. The first color in the name goes to the highest values, so high occupancy is red.
 3. Conditional Formatting → Manage Rules → Edit Rule shows Minimum = Lowest Value, Midpoint = Percentile 50, Maximum = Highest Value.
+4. Percentile 50 is the median, so the formula below gives the occupancy that gets pure yellow.
 Equivalent formula: =MEDIAN(Census!F2:F62)</t>
         </is>
       </c>
@@ -12398,11 +12411,11 @@
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>The 50th percentile is the median, the middle value when you sort the days by occupancy. Here 17 days have exactly that occupancy, so they show pure yellow. So the default color scale's middle color marks a typical day for this unit, not a target. To color against a target such as 85%, change the midpoint Type to Number (you'll do that in the bonus).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="186" customHeight="1">
+          <t>The 50th percentile is the median, the middle value when you sort the days by occupancy. Here 17 days have exactly that occupancy, so they all show pure yellow. The default color scale's middle color therefore marks a typical day for this unit, not a target. To color against a target such as 85%, change the midpoint Type to Number (you'll do that in the bonus).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="246" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>11</t>
@@ -12410,7 +12423,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Labs, TATMin: apply Icon Sets → 3 Traffic Lights (Unrimmed). Edit the rule: click Reverse Icon Order, set both Types to Number, and make red show when the value is &gt;= 60 and yellow when it is &gt;= 45 (green below 45). How many cells show a yellow light?</t>
+          <t>Labs, TATMin (L2:L322): apply Icon Sets → 3 Traffic Lights (Unrimmed). Edit the rule: click Reverse Icon Order, set both Types to Number, and make red show when the value is &gt;= 60 and yellow when it is &gt;= 45 (green below 45). How many cells show a yellow light?</t>
         </is>
       </c>
       <c r="C15" s="45" t="n">
@@ -12421,6 +12434,7 @@
           <t>1. Select L2:L322 → Home → Conditional Formatting → Icon Sets → 3 Traffic Lights (Unrimmed).
 2. Manage Rules → Edit Rule. Click Reverse Icon Order so red is on top.
 3. Red: &gt;=, Value 60, Type Number. Yellow: &gt;=, Value 45, Type Number. Green covers everything below 45. Click OK twice.
+4. Click the TATMin filter arrow → Filter by Color → Filter by Cell Icon → the yellow light, and read the count on the status bar: 79. Clear the filter afterward.
 Equivalent formula: =COUNTIFS(Labs!L2:L322,"&gt;=45",Labs!L2:L322,"&lt;60")</t>
         </is>
       </c>
@@ -12434,7 +12448,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="186" customHeight="1">
+    <row r="16" ht="231" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>12</t>
@@ -12453,6 +12467,7 @@
           <t>1. On Labs, type A2:L322 in the Name Box and press Enter. The rows are selected and A2 is the active cell.
 2. Home → Conditional Formatting → New Rule → Use a formula to determine which cells to format.
 3. Formula: =OR($K2="HH",$K2="LL"). Click Format → Fill, pick red, then OK twice.
+4. Filter any column from B to K by that red fill (no earlier rule colors those columns) and read the count on the status bar: 14.
 Equivalent formula: =COUNTIF(Labs!K2:K322,"HH")+COUNTIF(Labs!K2:K322,"LL")</t>
         </is>
       </c>
@@ -12466,7 +12481,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="291" customHeight="1">
+    <row r="17" ht="321" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
           <t>13</t>
@@ -12486,6 +12501,7 @@
 2. New Rule → Use a formula: =AND($L2&lt;&gt;"",$L2&lt;=ReportDate) with a red fill → OK.
 3. With the same range selected, add a second rule: =AND($L2&lt;&gt;"",$L2&lt;=ReportDate+ExpiringWindowDays) with an amber (light orange) fill → OK.
 4. Conditional Formatting → Manage Rules, set Show formatting rules for: This Worksheet. The amber rule is on top because Excel adds each new rule at the top of the list. Select the red rule and click ▲ (Move Up) so it sits above the amber rule, then click OK.
+5. Filter column A by the amber fill and read the count on the status bar: 7.
 Equivalent formula: =COUNTIFS(Supplies!L2:L258,"&gt;"&amp;ReportDate,Supplies!L2:L258,"&lt;="&amp;ReportDate+ExpiringWindowDays)</t>
         </is>
       </c>
@@ -12580,7 +12596,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Apply a 3-color scale to Occupancy (G12:G29): Minimum = Lowest Value (green), Midpoint = Number 0.85 (yellow, the planning target), Maximum = Highest Value (red). How many units are shaded on the red side of yellow (occupancy above 85%)?</t>
+          <t>On Huddle, apply a 3-color scale to Occupancy (G12:G29): Minimum = Lowest Value (green), Midpoint = Number 0.85 (yellow, the planning target), Maximum = Highest Value (red). How many units are shaded on the red side of yellow (occupancy above 85%)?</t>
         </is>
       </c>
       <c r="C5" s="45" t="n">
@@ -12611,7 +12627,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Apply Icon Sets → 3 Arrows (Colored) to Change (F12:F29). Edit the rule so both Types are Number: up arrow when the value is &gt;= 1, sideways arrow when it is &gt;= 0, down arrow otherwise. How many units show an up arrow?</t>
+          <t>On Huddle, apply Icon Sets → 3 Arrows (Colored) to Change (F12:F29). Edit the rule so both Types are Number: up arrow when the value is &gt;= 1, sideways arrow when it is &gt;= 0, down arrow otherwise. How many units show an up arrow?</t>
         </is>
       </c>
       <c r="C6" s="45" t="n">
@@ -12642,7 +12658,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Add two formula rules to the whole board (A12:G29): a red fill when the 11/25 census is above staffed beds (overflow), and an amber fill when occupancy is at least 90%. In Manage Rules, put the overflow rule above the amber rule. How many rows end up amber?</t>
+          <t>On Huddle, add two formula rules to the whole board (A12:G29): a red fill when the 11/25 census is above staffed beds (overflow), and an amber fill when occupancy is at least 90%. In Manage Rules, put the overflow rule above the amber rule. How many rows end up amber?</t>
         </is>
       </c>
       <c r="C7" s="45" t="n">
@@ -12667,7 +12683,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="381" customHeight="1">
+    <row r="8" ht="409" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>B4</t>
@@ -12675,7 +12691,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Build the unit selector. Give B4 a List validation from the Hospitals list (I12:I14). Give B5 a dependent List built from the board's own Facility and Unit columns, with no named ranges. Then choose Cedar Ridge Medical Center → Intensive Care Unit. The gray cell shows the card's Nov 1–25 occupancy. What is it?</t>
+          <t>On Huddle, build the unit selector. Give B4 a List validation from the Hospitals list (I12:I14). Give B5 a dependent List built from the board's own Facility and Unit columns, with no named ranges. Then pick Cedar Ridge Medical Center in B4 and Intensive Care Unit in B5. The gray answer cell on the Bonus sheet copies the card's Nov 1–25 occupancy (Huddle!B8), so it fills in and turns ✔ when your selector works.</t>
         </is>
       </c>
       <c r="C8" s="48" t="n">
@@ -12686,9 +12702,10 @@
           <t>1. Select B4 on Huddle → Data Validation → List, Source =$I$12:$I$14.
 2. Select B5 → Data Validation → List, Source:
    =OFFSET($B$11,MATCH($B$4,$A$12:$A$29,0),0,COUNTIF($A$12:$A$29,$B$4),1)
-   MATCH finds the facility's first row on the board, and COUNTIF counts its units. The board is sorted by facility, so OFFSET returns exactly that facility's block of unit names. If B4 is still empty, Excel warns that the source currently evaluates to an error. Click Yes, or pick a facility in B4 first.
-3. Pick Cedar Ridge Medical Center in B4, then Intensive Care Unit in B5. Read the card.
-If you prefer INDIRECT, copy each hospital's units into its own column under the hospital's name (like the Lists sheet in task 6), name the columns with Create from Selection, and use =INDIRECT(SUBSTITUTE($B$4," ","_")). The result is the same.</t>
+   MATCH finds the facility's first row on the board, and COUNTIF counts its units. The board lists each facility's units together, so OFFSET returns exactly that facility's block of unit names. If B4 is still empty, Excel warns that the source currently evaluates to an error. Click Yes, or pick a facility in B4 first.
+3. Pick Cedar Ridge Medical Center in B4, then Intensive Care Unit in B5. The card fills in, and the gray answer cell on the Bonus sheet shows its occupancy.
+The guide's version starts at Lists!K1 and uses $H2, because every intake row has its own facility. Here the start is the board's Unit header (B11) and the parent is the single cell $B$4.
+An INDIRECT version would need a second set of named lists that hold only the inpatient units. The names from task 6 (such as Cedar_Ridge_Medical_Center) already point at every department on the Lists sheet, so new names would have to differ from them. OFFSET skips that setup because it reads the board itself.</t>
         </is>
       </c>
       <c r="E8" cm="1" s="49">
@@ -12697,7 +12714,7 @@
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>Three hospitals each have an Intensive Care Unit, so the unit name alone is ambiguous. The dependent list forces a facility first and then offers only that facility's units, and the card's SUMIFS uses both cells. The OFFSET version needs no named ranges, so it keeps working when you add a unit to the board (as long as the board stays sorted by facility).</t>
+          <t>Three hospitals each have an Intensive Care Unit, so the unit name alone is ambiguous. The dependent list forces a facility first and then offers only that facility's units, and the card's SUMIFS uses both cells. The OFFSET version needs no named ranges. If you insert a new unit's row inside its facility's block, the board ranges in the formula grow to include it, so the list keeps working.</t>
         </is>
       </c>
     </row>
@@ -13675,7 +13692,7 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Labs, TATMin (L2:L322): turnaround minutes from specimen collection to result. Apply Top/Bottom Rules → Top 10 Items. What is the smallest TAT that your rule highlights?</t>
+          <t>Labs, TATMin (L2:L322): turnaround minutes from specimen collection to result. Apply Top/Bottom Rules → Top 10 Items. What is the smallest TAT that your rule highlights? Enter it in minutes.</t>
         </is>
       </c>
       <c r="C13" s="20" t="inlineStr">
@@ -13689,7 +13706,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="51" customHeight="1">
+    <row r="14" ht="66" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>9</t>
@@ -13697,12 +13714,12 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Supplies, PctOfPar (K2:K258) = QtyOnHand ÷ ParLevel. Add Data Bars, then edit the rule so Minimum is Number 0 and Maximum is Number 1. A full bar now means "stocked to par." How many items show a completely full bar?</t>
+          <t>Supplies, PctOfPar (K2:K258) is QtyOnHand ÷ ParLevel. Add Data Bars, then edit the rule so Minimum is Type Number, Value 0 and Maximum is Type Number, Value 1. A full bar now means "stocked to par or above." How many items show a full bar?</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
         <is>
-          <t>Values at or above the Maximum get a full bar</t>
+          <t>Every value at or above the Maximum gets a full bar. Filter by Color can't see bars, but COUNTIF can count them</t>
         </is>
       </c>
       <c r="D14" s="21" t="n"/>
@@ -13741,12 +13758,12 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Labs, TATMin: apply Icon Sets → 3 Traffic Lights (Unrimmed). Edit the rule: click Reverse Icon Order, set both Types to Number, and make red show when the value is &gt;= 60 and yellow when it is &gt;= 45 (green below 45). How many cells show a yellow light?</t>
+          <t>Labs, TATMin (L2:L322): apply Icon Sets → 3 Traffic Lights (Unrimmed). Edit the rule: click Reverse Icon Order, set both Types to Number, and make red show when the value is &gt;= 60 and yellow when it is &gt;= 45 (green below 45). How many cells show a yellow light?</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>Each icon's test is "&gt;=". The default Type is Percent, not Number</t>
+          <t>Each icon's test is "&gt;=". The default Type is Percent, not Number. Filter by Color → Filter by Cell Icon counts icons</t>
         </is>
       </c>
       <c r="D16" s="21" t="n"/>
@@ -16720,7 +16737,7 @@
     <row r="34">
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>The same pairs in long form (used by the answer key's check formula).</t>
+          <t>The same pairs in long form, grouped by facility (used by the guide's OFFSET example and the answer key's check formula).</t>
         </is>
       </c>
     </row>
@@ -48719,7 +48736,7 @@
     <row r="2" ht="64" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>It's 7 a.m. on Wednesday, November 26, 2025, the day before Thanksgiving. The house supervisor runs the system bed huddle from the Huddle sheet: one row per inpatient unit, with the midnight census for 11/24 and 11/25, the overnight change, and occupancy. Make the board readable at a glance, then build the unit selector that drives the gray unit card (B6:B9). The card reads the NovCensus sheet (every unit, Nov 1–25). The board's data is in rows 12–29.</t>
+          <t>It's 7 a.m. on Wednesday, November 26, 2025, the day before Thanksgiving. The house supervisor runs the system bed huddle from the Huddle sheet: one row per inpatient unit, with the midnight census for 11/24 and 11/25, the overnight change, and occupancy. Make the board readable at a glance, then build the unit selector that drives the gray unit card (Huddle!B6:B9). The card reads the NovCensus sheet (every unit, Nov 1–25). The board's data is in rows 12–29. Build every rule and the selector on the Huddle sheet, and type your answers on the Bonus sheet.</t>
         </is>
       </c>
     </row>
@@ -48771,7 +48788,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Apply a 3-color scale to Occupancy (G12:G29): Minimum = Lowest Value (green), Midpoint = Number 0.85 (yellow, the planning target), Maximum = Highest Value (red). How many units are shaded on the red side of yellow (occupancy above 85%)?</t>
+          <t>On Huddle, apply a 3-color scale to Occupancy (G12:G29): Minimum = Lowest Value (green), Midpoint = Number 0.85 (yellow, the planning target), Maximum = Highest Value (red). How many units are shaded on the red side of yellow (occupancy above 85%)?</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -48793,7 +48810,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Apply Icon Sets → 3 Arrows (Colored) to Change (F12:F29). Edit the rule so both Types are Number: up arrow when the value is &gt;= 1, sideways arrow when it is &gt;= 0, down arrow otherwise. How many units show an up arrow?</t>
+          <t>On Huddle, apply Icon Sets → 3 Arrows (Colored) to Change (F12:F29). Edit the rule so both Types are Number: up arrow when the value is &gt;= 1, sideways arrow when it is &gt;= 0, down arrow otherwise. How many units show an up arrow?</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -48815,7 +48832,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Add two formula rules to the whole board (A12:G29): a red fill when the 11/25 census is above staffed beds (overflow), and an amber fill when occupancy is at least 90%. In Manage Rules, put the overflow rule above the amber rule. How many rows end up amber?</t>
+          <t>On Huddle, add two formula rules to the whole board (A12:G29): a red fill when the 11/25 census is above staffed beds (overflow), and an amber fill when occupancy is at least 90%. In Manage Rules, put the overflow rule above the amber rule. How many rows end up amber?</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -48829,7 +48846,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="66" customHeight="1">
+    <row r="9" ht="96" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>B4</t>
@@ -48837,12 +48854,12 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Build the unit selector. Give B4 a List validation from the Hospitals list (I12:I14). Give B5 a dependent List built from the board's own Facility and Unit columns, with no named ranges. Then choose Cedar Ridge Medical Center → Intensive Care Unit. The gray cell shows the card's Nov 1–25 occupancy. What is it?</t>
+          <t>On Huddle, build the unit selector. Give B4 a List validation from the Hospitals list (I12:I14). Give B5 a dependent List built from the board's own Facility and Unit columns, with no named ranges. Then pick Cedar Ridge Medical Center in B4 and Intensive Care Unit in B5. The gray answer cell on the Bonus sheet copies the card's Nov 1–25 occupancy (Huddle!B8), so it fills in and turns ✔ when your selector works.</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>OFFSET(start, rows down, 0, height, 1) with MATCH for the first row and COUNTIF for the height</t>
+          <t>Adapt the OFFSET example in guide section 6: MATCH finds the facility's first row and COUNTIF its height</t>
         </is>
       </c>
       <c r="D9" cm="1" s="33">

</xml_diff>